<commit_message>
changes to plotting function to compare HH to FT predictions
</commit_message>
<xml_diff>
--- a/+Farrell2024/+data/PreObsFilmThicknessComparison.xlsx
+++ b/+Farrell2024/+data/PreObsFilmThicknessComparison.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uwprod-my.sharepoint.com/personal/tlee239_wisc_edu/Documents/Documents/01_Research/01_OpenSTREAM/GitHub/openstream-database/+Farrell2024/+data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="58" documentId="8_{634B5368-7D98-4999-AD8C-8076C34C5E2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2B68DFC6-FB87-4EC7-9BCB-8F35022847D5}"/>
+  <xr:revisionPtr revIDLastSave="99" documentId="8_{634B5368-7D98-4999-AD8C-8076C34C5E2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E1046C75-8E64-432E-B760-BDD0A3B1ADE5}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{4592F272-D649-4DC6-BAB0-584D00ED6D07}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4592F272-D649-4DC6-BAB0-584D00ED6D07}"/>
   </bookViews>
   <sheets>
     <sheet name="PreObsFilmThicknessComparison" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="77">
   <si>
     <t>Param Name</t>
   </si>
@@ -258,6 +258,15 @@
   </si>
   <si>
     <t>[0.096]</t>
+  </si>
+  <si>
+    <t>weightedAvgFT [m]</t>
+  </si>
+  <si>
+    <t>timeAvgFT [m]</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -1119,28 +1128,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4329B02C-9C1B-4A7A-8D40-84ADEA2A1E65}">
-  <dimension ref="A1:O56"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:R63"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.6328125" customWidth="1"/>
-    <col min="2" max="2" width="22.6328125" customWidth="1"/>
-    <col min="3" max="3" width="22.36328125" customWidth="1"/>
-    <col min="4" max="4" width="27.26953125" customWidth="1"/>
-    <col min="5" max="5" width="27.36328125" customWidth="1"/>
-    <col min="6" max="6" width="42.36328125" customWidth="1"/>
-    <col min="7" max="7" width="39.90625" customWidth="1"/>
-    <col min="8" max="8" width="13.90625" customWidth="1"/>
-    <col min="9" max="9" width="17.26953125" customWidth="1"/>
-    <col min="10" max="10" width="16.90625" customWidth="1"/>
-    <col min="11" max="11" width="14.7265625" customWidth="1"/>
+    <col min="1" max="1" width="24.5703125" customWidth="1"/>
+    <col min="2" max="2" width="22.5703125" customWidth="1"/>
+    <col min="3" max="3" width="22.42578125" customWidth="1"/>
+    <col min="4" max="4" width="27.28515625" customWidth="1"/>
+    <col min="5" max="5" width="27.42578125" customWidth="1"/>
+    <col min="6" max="6" width="42.42578125" customWidth="1"/>
+    <col min="7" max="7" width="39.85546875" customWidth="1"/>
+    <col min="8" max="8" width="13.85546875" customWidth="1"/>
+    <col min="9" max="9" width="17.28515625" customWidth="1"/>
+    <col min="10" max="10" width="16.85546875" customWidth="1"/>
+    <col min="11" max="11" width="14.7109375" customWidth="1"/>
     <col min="12" max="12" width="17" customWidth="1"/>
-    <col min="13" max="13" width="17.90625" customWidth="1"/>
-    <col min="14" max="14" width="10.26953125" customWidth="1"/>
-    <col min="15" max="15" width="26.6328125" customWidth="1"/>
-    <col min="16" max="16" width="21.90625" customWidth="1"/>
+    <col min="13" max="13" width="17.85546875" customWidth="1"/>
+    <col min="14" max="14" width="10.28515625" customWidth="1"/>
+    <col min="15" max="16" width="30.42578125" customWidth="1"/>
+    <col min="17" max="17" width="20.42578125" customWidth="1"/>
+    <col min="18" max="18" width="24.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1186,8 +1196,14 @@
       <c r="O1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q1" t="s">
+        <v>74</v>
+      </c>
+      <c r="R1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -1234,8 +1250,14 @@
       <c r="O2">
         <v>1.6539500000000001E-4</v>
       </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q2">
+        <v>2.015919E-4</v>
+      </c>
+      <c r="R2">
+        <v>1.6539500000000001E-4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -1254,8 +1276,8 @@
       <c r="F3" s="1">
         <v>12870</v>
       </c>
-      <c r="G3">
-        <f t="shared" si="0"/>
+      <c r="G3" s="1">
+        <f>F3*I3*0.036*2</f>
         <v>373.43592000000001</v>
       </c>
       <c r="H3">
@@ -1282,8 +1304,14 @@
       <c r="O3">
         <v>1.4779100000000001E-4</v>
       </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q3">
+        <v>1.8023259999999999E-4</v>
+      </c>
+      <c r="R3">
+        <v>1.4779100000000001E-4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -1330,8 +1358,14 @@
       <c r="O4">
         <v>1.40586E-4</v>
       </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q4">
+        <v>1.7355989999999998E-4</v>
+      </c>
+      <c r="R4">
+        <v>1.40586E-4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1378,8 +1412,14 @@
       <c r="O5">
         <v>1.28319E-4</v>
       </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q5">
+        <v>1.593377E-4</v>
+      </c>
+      <c r="R5">
+        <v>1.28319E-4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -1426,8 +1466,14 @@
       <c r="O6">
         <v>1.36508E-4</v>
       </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q6">
+        <v>1.6810300000000001E-4</v>
+      </c>
+      <c r="R6">
+        <v>1.36508E-4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -1474,8 +1520,14 @@
       <c r="O7">
         <v>1.1874E-4</v>
       </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q7">
+        <v>1.463638E-4</v>
+      </c>
+      <c r="R7">
+        <v>1.1874E-4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>20</v>
       </c>
@@ -1522,8 +1574,14 @@
       <c r="O8">
         <v>1.17469E-4</v>
       </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q8">
+        <v>1.4332099999999999E-4</v>
+      </c>
+      <c r="R8">
+        <v>1.17469E-4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -1570,8 +1628,14 @@
       <c r="O9">
         <v>1.12574E-4</v>
       </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q9">
+        <v>1.3998259999999999E-4</v>
+      </c>
+      <c r="R9">
+        <v>1.12574E-4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1618,8 +1682,14 @@
       <c r="O10">
         <v>1.17737E-4</v>
       </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q10">
+        <v>1.3968419999999999E-4</v>
+      </c>
+      <c r="R10">
+        <v>1.17737E-4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -1666,8 +1736,14 @@
       <c r="O11">
         <v>1.00109E-4</v>
       </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q11">
+        <v>1.262852E-4</v>
+      </c>
+      <c r="R11">
+        <v>1.00109E-4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>24</v>
       </c>
@@ -1714,8 +1790,15 @@
       <c r="O12" s="1">
         <v>9.5099999999999994E-5</v>
       </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P12" s="1"/>
+      <c r="Q12">
+        <v>1.1961549999999999E-4</v>
+      </c>
+      <c r="R12" s="1">
+        <v>9.5099999999999994E-5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -1762,8 +1845,15 @@
       <c r="O13" s="1">
         <v>9.4300000000000002E-5</v>
       </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P13" s="1"/>
+      <c r="Q13">
+        <v>1.1740579999999999E-4</v>
+      </c>
+      <c r="R13" s="1">
+        <v>9.4300000000000002E-5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>26</v>
       </c>
@@ -1810,8 +1900,15 @@
       <c r="O14" s="1">
         <v>9.5400000000000001E-5</v>
       </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P14" s="1"/>
+      <c r="Q14">
+        <v>1.1935489999999999E-4</v>
+      </c>
+      <c r="R14" s="1">
+        <v>9.5400000000000001E-5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>27</v>
       </c>
@@ -1858,8 +1955,15 @@
       <c r="O15" s="1">
         <v>7.9599999999999997E-5</v>
       </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P15" s="1"/>
+      <c r="Q15">
+        <v>9.8605599999999997E-5</v>
+      </c>
+      <c r="R15" s="1">
+        <v>7.9599999999999997E-5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>28</v>
       </c>
@@ -1906,8 +2010,15 @@
       <c r="O16" s="1">
         <v>6.8999999999999997E-5</v>
       </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P16" s="1"/>
+      <c r="Q16">
+        <v>9.4988999999999995E-5</v>
+      </c>
+      <c r="R16" s="1">
+        <v>6.8999999999999997E-5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>29</v>
       </c>
@@ -1954,8 +2065,15 @@
       <c r="O17" s="1">
         <v>6.3899999999999995E-5</v>
       </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P17" s="1"/>
+      <c r="Q17">
+        <v>9.3033099999999995E-5</v>
+      </c>
+      <c r="R17" s="1">
+        <v>6.3899999999999995E-5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>30</v>
       </c>
@@ -2002,8 +2120,14 @@
       <c r="O18">
         <v>1.59369E-4</v>
       </c>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q18">
+        <v>1.9306559999999998E-4</v>
+      </c>
+      <c r="R18">
+        <v>1.59369E-4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>31</v>
       </c>
@@ -2050,8 +2174,14 @@
       <c r="O19">
         <v>1.4241500000000001E-4</v>
       </c>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q19">
+        <v>1.7401910000000001E-4</v>
+      </c>
+      <c r="R19">
+        <v>1.4241500000000001E-4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>32</v>
       </c>
@@ -2098,8 +2228,14 @@
       <c r="O20">
         <v>1.29309E-4</v>
       </c>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q20">
+        <v>1.6080469999999998E-4</v>
+      </c>
+      <c r="R20">
+        <v>1.29309E-4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>33</v>
       </c>
@@ -2146,8 +2282,14 @@
       <c r="O21">
         <v>1.2746E-4</v>
       </c>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q21">
+        <v>1.5574129999999998E-4</v>
+      </c>
+      <c r="R21">
+        <v>1.2746E-4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>34</v>
       </c>
@@ -2194,8 +2336,14 @@
       <c r="O22">
         <v>1.39622E-4</v>
       </c>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q22">
+        <v>1.7095670000000002E-4</v>
+      </c>
+      <c r="R22">
+        <v>1.39622E-4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>35</v>
       </c>
@@ -2242,8 +2390,14 @@
       <c r="O23">
         <v>1.1931500000000001E-4</v>
       </c>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q23">
+        <v>1.4414519999999997E-4</v>
+      </c>
+      <c r="R23">
+        <v>1.1931500000000001E-4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>36</v>
       </c>
@@ -2290,8 +2444,14 @@
       <c r="O24">
         <v>1.14428E-4</v>
       </c>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q24">
+        <v>1.4025409999999998E-4</v>
+      </c>
+      <c r="R24">
+        <v>1.14428E-4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>37</v>
       </c>
@@ -2338,8 +2498,14 @@
       <c r="O25">
         <v>1.20362E-4</v>
       </c>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q25">
+        <v>1.4262079999999999E-4</v>
+      </c>
+      <c r="R25">
+        <v>1.20362E-4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>38</v>
       </c>
@@ -2386,8 +2552,14 @@
       <c r="O26">
         <v>1.0671E-4</v>
       </c>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q26">
+        <v>1.289435E-4</v>
+      </c>
+      <c r="R26">
+        <v>1.0671E-4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>39</v>
       </c>
@@ -2434,8 +2606,15 @@
       <c r="O27" s="1">
         <v>9.7600000000000001E-5</v>
       </c>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P27" s="1"/>
+      <c r="Q27">
+        <v>1.169535E-4</v>
+      </c>
+      <c r="R27" s="1">
+        <v>9.7600000000000001E-5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>40</v>
       </c>
@@ -2482,8 +2661,15 @@
       <c r="O28" s="1">
         <v>9.6100000000000005E-5</v>
       </c>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P28" s="1"/>
+      <c r="Q28">
+        <v>1.157346E-4</v>
+      </c>
+      <c r="R28" s="1">
+        <v>9.6100000000000005E-5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>41</v>
       </c>
@@ -2530,8 +2716,14 @@
       <c r="O29">
         <v>1.0501300000000001E-4</v>
       </c>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q29">
+        <v>1.2519199999999999E-4</v>
+      </c>
+      <c r="R29">
+        <v>1.0501300000000001E-4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>42</v>
       </c>
@@ -2578,8 +2770,15 @@
       <c r="O30" s="1">
         <v>9.2100000000000003E-5</v>
       </c>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P30" s="1"/>
+      <c r="Q30">
+        <v>1.116945E-4</v>
+      </c>
+      <c r="R30" s="1">
+        <v>9.2100000000000003E-5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>43</v>
       </c>
@@ -2626,8 +2825,15 @@
       <c r="O31" s="1">
         <v>8.8300000000000005E-5</v>
       </c>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P31" s="1"/>
+      <c r="Q31">
+        <v>1.0675559999999999E-4</v>
+      </c>
+      <c r="R31" s="1">
+        <v>8.8300000000000005E-5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>44</v>
       </c>
@@ -2674,8 +2880,15 @@
       <c r="O32" s="1">
         <v>8.2100000000000003E-5</v>
       </c>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P32" s="1"/>
+      <c r="Q32">
+        <v>9.9657499999999992E-5</v>
+      </c>
+      <c r="R32" s="1">
+        <v>8.2100000000000003E-5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>45</v>
       </c>
@@ -2722,8 +2935,15 @@
       <c r="O33" s="1">
         <v>8.3800000000000004E-5</v>
       </c>
-    </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P33" s="1"/>
+      <c r="Q33">
+        <v>9.9484899999999993E-5</v>
+      </c>
+      <c r="R33" s="1">
+        <v>8.3800000000000004E-5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>46</v>
       </c>
@@ -2770,8 +2990,15 @@
       <c r="O34" s="1">
         <v>8.1899999999999999E-5</v>
       </c>
-    </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P34" s="1"/>
+      <c r="Q34">
+        <v>9.7251599999999996E-5</v>
+      </c>
+      <c r="R34" s="1">
+        <v>8.1899999999999999E-5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>47</v>
       </c>
@@ -2818,8 +3045,15 @@
       <c r="O35" s="1">
         <v>7.0400000000000004E-5</v>
       </c>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P35" s="1"/>
+      <c r="Q35">
+        <v>8.6312700000000005E-5</v>
+      </c>
+      <c r="R35" s="1">
+        <v>7.0400000000000004E-5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>48</v>
       </c>
@@ -2866,8 +3100,15 @@
       <c r="O36" s="1">
         <v>7.0099999999999996E-5</v>
       </c>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P36" s="1"/>
+      <c r="Q36">
+        <v>8.7439499999999995E-5</v>
+      </c>
+      <c r="R36" s="1">
+        <v>7.0099999999999996E-5</v>
+      </c>
+    </row>
+    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>49</v>
       </c>
@@ -2914,8 +3155,14 @@
       <c r="O37">
         <v>1.47186E-4</v>
       </c>
-    </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q37">
+        <v>1.8173159999999999E-4</v>
+      </c>
+      <c r="R37">
+        <v>1.47186E-4</v>
+      </c>
+    </row>
+    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>50</v>
       </c>
@@ -2962,8 +3209,14 @@
       <c r="O38">
         <v>1.28665E-4</v>
       </c>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q38">
+        <v>1.5544059999999998E-4</v>
+      </c>
+      <c r="R38">
+        <v>1.28665E-4</v>
+      </c>
+    </row>
+    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>51</v>
       </c>
@@ -3010,8 +3263,14 @@
       <c r="O39">
         <v>1.11675E-4</v>
       </c>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q39">
+        <v>1.3881589999999999E-4</v>
+      </c>
+      <c r="R39">
+        <v>1.11675E-4</v>
+      </c>
+    </row>
+    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>52</v>
       </c>
@@ -3058,8 +3317,14 @@
       <c r="O40">
         <v>1.0819699999999999E-4</v>
       </c>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q40">
+        <v>1.3615249999999999E-4</v>
+      </c>
+      <c r="R40">
+        <v>1.0819699999999999E-4</v>
+      </c>
+    </row>
+    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>53</v>
       </c>
@@ -3106,8 +3371,14 @@
       <c r="O41">
         <v>1.2542900000000001E-4</v>
       </c>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q41">
+        <v>1.5256769999999999E-4</v>
+      </c>
+      <c r="R41">
+        <v>1.2542900000000001E-4</v>
+      </c>
+    </row>
+    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>54</v>
       </c>
@@ -3154,8 +3425,14 @@
       <c r="O42">
         <v>1.13292E-4</v>
       </c>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q42">
+        <v>1.3753389999999999E-4</v>
+      </c>
+      <c r="R42">
+        <v>1.13292E-4</v>
+      </c>
+    </row>
+    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>55</v>
       </c>
@@ -3202,8 +3479,14 @@
       <c r="O43">
         <v>1.0514E-4</v>
       </c>
-    </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q43">
+        <v>1.2954349999999998E-4</v>
+      </c>
+      <c r="R43">
+        <v>1.0514E-4</v>
+      </c>
+    </row>
+    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>56</v>
       </c>
@@ -3250,8 +3533,14 @@
       <c r="O44">
         <v>1.0189200000000001E-4</v>
       </c>
-    </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q44">
+        <v>1.2787789999999999E-4</v>
+      </c>
+      <c r="R44">
+        <v>1.0189200000000001E-4</v>
+      </c>
+    </row>
+    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>57</v>
       </c>
@@ -3298,8 +3587,14 @@
       <c r="O45">
         <v>1.08825E-4</v>
       </c>
-    </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="Q45">
+        <v>1.3133940000000001E-4</v>
+      </c>
+      <c r="R45">
+        <v>1.08825E-4</v>
+      </c>
+    </row>
+    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>58</v>
       </c>
@@ -3346,8 +3641,15 @@
       <c r="O46" s="1">
         <v>9.7499999999999998E-5</v>
       </c>
-    </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P46" s="1"/>
+      <c r="Q46">
+        <v>1.1698929999999999E-4</v>
+      </c>
+      <c r="R46" s="1">
+        <v>9.7499999999999998E-5</v>
+      </c>
+    </row>
+    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>59</v>
       </c>
@@ -3394,8 +3696,15 @@
       <c r="O47" s="1">
         <v>9.2E-5</v>
       </c>
-    </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P47" s="1"/>
+      <c r="Q47">
+        <v>1.104161E-4</v>
+      </c>
+      <c r="R47" s="1">
+        <v>9.2E-5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>60</v>
       </c>
@@ -3442,8 +3751,15 @@
       <c r="O48" s="1">
         <v>9.0500000000000004E-5</v>
       </c>
-    </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P48" s="1"/>
+      <c r="Q48">
+        <v>1.094509E-4</v>
+      </c>
+      <c r="R48" s="1">
+        <v>9.0500000000000004E-5</v>
+      </c>
+    </row>
+    <row r="49" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>61</v>
       </c>
@@ -3490,8 +3806,15 @@
       <c r="O49" s="1">
         <v>9.4900000000000003E-5</v>
       </c>
-    </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P49" s="1"/>
+      <c r="Q49">
+        <v>1.1298869999999999E-4</v>
+      </c>
+      <c r="R49" s="1">
+        <v>9.4900000000000003E-5</v>
+      </c>
+    </row>
+    <row r="50" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>62</v>
       </c>
@@ -3538,8 +3861,15 @@
       <c r="O50" s="1">
         <v>8.6899999999999998E-5</v>
       </c>
-    </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P50" s="1"/>
+      <c r="Q50">
+        <v>1.0275149999999999E-4</v>
+      </c>
+      <c r="R50" s="1">
+        <v>8.6899999999999998E-5</v>
+      </c>
+    </row>
+    <row r="51" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>63</v>
       </c>
@@ -3586,8 +3916,15 @@
       <c r="O51" s="1">
         <v>8.4499999999999994E-5</v>
       </c>
-    </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P51" s="1"/>
+      <c r="Q51">
+        <v>1.00571E-4</v>
+      </c>
+      <c r="R51" s="1">
+        <v>8.4499999999999994E-5</v>
+      </c>
+    </row>
+    <row r="52" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>64</v>
       </c>
@@ -3634,8 +3971,15 @@
       <c r="O52" s="1">
         <v>8.1899999999999999E-5</v>
       </c>
-    </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P52" s="1"/>
+      <c r="Q52">
+        <v>9.7030100000000005E-5</v>
+      </c>
+      <c r="R52" s="1">
+        <v>8.1899999999999999E-5</v>
+      </c>
+    </row>
+    <row r="53" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>65</v>
       </c>
@@ -3682,8 +4026,15 @@
       <c r="O53" s="1">
         <v>8.1299999999999997E-5</v>
       </c>
-    </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P53" s="1"/>
+      <c r="Q53">
+        <v>9.5344699999999995E-5</v>
+      </c>
+      <c r="R53" s="1">
+        <v>8.1299999999999997E-5</v>
+      </c>
+    </row>
+    <row r="54" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>66</v>
       </c>
@@ -3730,8 +4081,15 @@
       <c r="O54" s="1">
         <v>7.7700000000000005E-5</v>
       </c>
-    </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P54" s="1"/>
+      <c r="Q54">
+        <v>9.0803200000000005E-5</v>
+      </c>
+      <c r="R54" s="1">
+        <v>7.7700000000000005E-5</v>
+      </c>
+    </row>
+    <row r="55" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>67</v>
       </c>
@@ -3778,8 +4136,15 @@
       <c r="O55" s="1">
         <v>7.2999999999999999E-5</v>
       </c>
-    </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P55" s="1"/>
+      <c r="Q55">
+        <v>8.517199999999999E-5</v>
+      </c>
+      <c r="R55" s="1">
+        <v>7.2999999999999999E-5</v>
+      </c>
+    </row>
+    <row r="56" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>68</v>
       </c>
@@ -3825,6 +4190,18 @@
       </c>
       <c r="O56" s="1">
         <v>6.6099999999999994E-5</v>
+      </c>
+      <c r="P56" s="1"/>
+      <c r="Q56">
+        <v>7.9966899999999995E-5</v>
+      </c>
+      <c r="R56" s="1">
+        <v>6.6099999999999994E-5</v>
+      </c>
+    </row>
+    <row r="63" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="Q63" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>